<commit_message>
resolved import for external call
</commit_message>
<xml_diff>
--- a/pythonWork/testModels/crmTest/DB/crmTest_datamodels.xlsx
+++ b/pythonWork/testModels/crmTest/DB/crmTest_datamodels.xlsx
@@ -436,12 +436,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,12 +454,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>tablecount</t>
+          <t>Tables</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>columncount</t>
+          <t>Enti/Rela mapped</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Columns</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Attributes mapped</t>
         </is>
       </c>
     </row>
@@ -471,7 +483,13 @@
         <v>46</v>
       </c>
       <c r="C2" t="n">
+        <v>45</v>
+      </c>
+      <c r="D2" t="n">
         <v>156</v>
+      </c>
+      <c r="E2" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -484,7 +502,13 @@
         <v>17</v>
       </c>
       <c r="C3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D3" t="n">
         <v>69</v>
+      </c>
+      <c r="E3" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -497,7 +521,13 @@
         <v>20</v>
       </c>
       <c r="C4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" t="n">
         <v>84</v>
+      </c>
+      <c r="E4" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -510,7 +540,13 @@
         <v>26</v>
       </c>
       <c r="C5" t="n">
+        <v>25</v>
+      </c>
+      <c r="D5" t="n">
         <v>95</v>
+      </c>
+      <c r="E5" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -523,7 +559,54 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
         <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Information Model</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Entities/Relations</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Tables mapped</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Attrbutes</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Columns-Mapped</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="n">
+        <v>43</v>
+      </c>
+      <c r="C9" t="n">
+        <v>109</v>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="n">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -4868,23 +4951,23 @@
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="35" customWidth="1" min="8" max="8"/>
     <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="35" customWidth="1" min="11" max="11"/>
     <col width="35" customWidth="1" min="12" max="12"/>
     <col width="5" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
     <col width="35" customWidth="1" min="15" max="15"/>
     <col width="35" customWidth="1" min="16" max="16"/>
     <col width="5" customWidth="1" min="17" max="17"/>
-    <col width="35" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
     <col width="35" customWidth="1" min="19" max="19"/>
     <col width="35" customWidth="1" min="20" max="20"/>
     <col width="5" customWidth="1" min="21" max="21"/>
-    <col width="35" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>